<commit_message>
updated purchasing data on 10th of may 2026 18.16
updated on 10th of may 2026 18.16
</commit_message>
<xml_diff>
--- a/FEBRUARY 2026/FLOOR FEBRUARY 2026.xlsx
+++ b/FEBRUARY 2026/FLOOR FEBRUARY 2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="16360" windowHeight="18640" firstSheet="1" activeTab="1"/>
+    <workbookView windowWidth="16120" windowHeight="18640" firstSheet="3" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Anugrah (Bag, Cup, Box)" sheetId="1" r:id="rId1"/>
@@ -31,12 +31,8 @@
 </workbook>
 </file>
 
-<file path=xl/cellimages.xml><?xml version="1.0" encoding="utf-8"?>
-<etc:cellImages xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData"/>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="67">
   <si>
     <t>DATE</t>
   </si>
@@ -167,13 +163,46 @@
     <t>SO05LC2602002826/00</t>
   </si>
   <si>
-    <t>STATUS</t>
+    <t>QTY</t>
+  </si>
+  <si>
+    <t>0201</t>
+  </si>
+  <si>
+    <t>0202</t>
+  </si>
+  <si>
+    <t>0203</t>
+  </si>
+  <si>
+    <t>0204</t>
+  </si>
+  <si>
+    <t>0205</t>
+  </si>
+  <si>
+    <t>0206</t>
+  </si>
+  <si>
+    <t>0207</t>
+  </si>
+  <si>
+    <t>0208</t>
+  </si>
+  <si>
+    <t>0209</t>
+  </si>
+  <si>
+    <t>0210</t>
+  </si>
+  <si>
+    <t>0211</t>
+  </si>
+  <si>
+    <t>0212</t>
   </si>
   <si>
     <t>DESCRIPTION</t>
-  </si>
-  <si>
-    <t>QTY</t>
   </si>
   <si>
     <t>DISHY 5 L DISHWASHIG</t>
@@ -210,7 +239,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
@@ -218,9 +247,10 @@
     <numFmt numFmtId="180" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="181" formatCode="[$-409]d\-mmm\-yyyy;@"/>
     <numFmt numFmtId="182" formatCode="[$Rp-421]#,##0.00;[Red][$Rp-421]#,##0.00"/>
-    <numFmt numFmtId="183" formatCode="dd\-mmm"/>
-    <numFmt numFmtId="184" formatCode="_ [$IDR]\ * #,##0_ ;_ [$IDR]\ * \-#,##0_ ;_ [$IDR]\ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="185" formatCode="[$Rp-421]#,##0.0000;[Red][$Rp-421]#,##0.0000"/>
+    <numFmt numFmtId="183" formatCode="0;[Red]0"/>
+    <numFmt numFmtId="184" formatCode="dd\-mmm"/>
+    <numFmt numFmtId="185" formatCode="_ [$IDR]\ * #,##0_ ;_ [$IDR]\ * \-#,##0_ ;_ [$IDR]\ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="186" formatCode="[$Rp-421]#,##0.0000;[Red][$Rp-421]#,##0.0000"/>
   </numFmts>
   <fonts count="33">
     <font>
@@ -1089,7 +1119,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1217,25 +1247,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="183" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="183" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="183" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="184" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="184" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="184" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="185" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1244,17 +1280,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1284,7 +1314,7 @@
     <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="183" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="184" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1320,28 +1350,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="185" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="186" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="182" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="185" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="185" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="186" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="186" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="182" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="185" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="185" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="186" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="186" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="185" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="186" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="180" fontId="8" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1522,13 +1555,13 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="184" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="184" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="184" fontId="9" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="185" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="9" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1542,6 +1575,9 @@
     </xf>
     <xf numFmtId="180" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1635,7 +1671,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7257415" y="230505"/>
+          <a:off x="6833870" y="230505"/>
           <a:ext cx="2531110" cy="3516630"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1674,7 +1710,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7263130" y="3786505"/>
+          <a:off x="6839585" y="3786505"/>
           <a:ext cx="2519680" cy="3517265"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2347,256 +2383,256 @@
   <dimension ref="A1:H12"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="20.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="17.4296875" style="98"/>
-    <col min="2" max="2" width="13.4296875" style="98" customWidth="1"/>
-    <col min="3" max="3" width="36" style="98" customWidth="1"/>
-    <col min="4" max="4" width="21.2890625" style="96" customWidth="1"/>
-    <col min="5" max="5" width="33.2890625" style="98" customWidth="1"/>
-    <col min="6" max="6" width="17.2890625" style="98" customWidth="1"/>
-    <col min="7" max="8" width="20.859375" style="98" customWidth="1"/>
-    <col min="9" max="9" width="12.859375" style="98"/>
-    <col min="10" max="10" width="15" style="98"/>
-    <col min="11" max="16384" width="18.0390625" style="98"/>
+    <col min="1" max="1" width="13.25" style="99" customWidth="1"/>
+    <col min="2" max="2" width="13.4296875" style="99" customWidth="1"/>
+    <col min="3" max="3" width="34.96875" style="99" customWidth="1"/>
+    <col min="4" max="4" width="21.2890625" style="97" customWidth="1"/>
+    <col min="5" max="5" width="33.2890625" style="99" customWidth="1"/>
+    <col min="6" max="6" width="17.2890625" style="99" customWidth="1"/>
+    <col min="7" max="8" width="20.859375" style="99" customWidth="1"/>
+    <col min="9" max="9" width="12.859375" style="99"/>
+    <col min="10" max="10" width="15" style="99"/>
+    <col min="11" max="16384" width="18.0390625" style="99"/>
   </cols>
   <sheetData>
-    <row r="1" s="94" customFormat="1" ht="16" customHeight="1" spans="1:8">
-      <c r="A1" s="147" t="s">
+    <row r="1" s="95" customFormat="1" ht="16" customHeight="1" spans="1:8">
+      <c r="A1" s="148" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="148" t="s">
+      <c r="B1" s="149" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="148" t="s">
+      <c r="C1" s="149" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="148" t="s">
+      <c r="D1" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="148" t="s">
+      <c r="E1" s="149" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="148" t="s">
+      <c r="F1" s="149" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="148" t="s">
+      <c r="G1" s="149" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="148" t="s">
+      <c r="H1" s="149" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="94" customFormat="1" ht="140" customHeight="1" spans="1:8">
-      <c r="A2" s="108">
+    <row r="2" s="95" customFormat="1" ht="140" customHeight="1" spans="1:8">
+      <c r="A2" s="109">
         <v>46056</v>
       </c>
-      <c r="B2" s="119">
+      <c r="B2" s="120">
         <v>3426</v>
       </c>
-      <c r="C2" s="149" t="s">
+      <c r="C2" s="150" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="150">
+      <c r="D2" s="151">
         <v>20</v>
       </c>
-      <c r="E2" s="132"/>
-      <c r="F2" s="154">
+      <c r="E2" s="133"/>
+      <c r="F2" s="155">
         <v>55000</v>
       </c>
-      <c r="G2" s="155">
+      <c r="G2" s="156">
         <f>SUM(D2*F2)</f>
         <v>1100000</v>
       </c>
-      <c r="H2" s="155">
+      <c r="H2" s="156">
         <f>SUM(G2:G3)</f>
         <v>1650000</v>
       </c>
     </row>
-    <row r="3" s="94" customFormat="1" ht="140" customHeight="1" spans="1:8">
-      <c r="A3" s="112"/>
-      <c r="B3" s="119"/>
-      <c r="C3" s="149" t="s">
+    <row r="3" s="95" customFormat="1" ht="140" customHeight="1" spans="1:8">
+      <c r="A3" s="113"/>
+      <c r="B3" s="120"/>
+      <c r="C3" s="150" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="150">
+      <c r="D3" s="151">
         <v>10</v>
       </c>
-      <c r="E3" s="136"/>
-      <c r="F3" s="154">
+      <c r="E3" s="137"/>
+      <c r="F3" s="155">
         <v>55000</v>
       </c>
-      <c r="G3" s="155">
+      <c r="G3" s="156">
         <f>SUM(D3*F3)</f>
         <v>550000</v>
       </c>
-      <c r="H3" s="156"/>
-    </row>
-    <row r="4" s="94" customFormat="1" ht="40" customHeight="1" spans="1:8">
-      <c r="A4" s="108">
+      <c r="H3" s="157"/>
+    </row>
+    <row r="4" s="95" customFormat="1" ht="40" customHeight="1" spans="1:8">
+      <c r="A4" s="109">
         <v>46058</v>
       </c>
-      <c r="B4" s="109">
+      <c r="B4" s="110">
         <v>3461</v>
       </c>
-      <c r="C4" s="151" t="s">
+      <c r="C4" s="152" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="150">
+      <c r="D4" s="151">
         <v>450</v>
       </c>
-      <c r="E4" s="132"/>
-      <c r="F4" s="155">
+      <c r="E4" s="133"/>
+      <c r="F4" s="156">
         <v>1800</v>
       </c>
-      <c r="G4" s="155">
+      <c r="G4" s="156">
         <f>SUM(D4*F4)</f>
         <v>810000</v>
       </c>
-      <c r="H4" s="155">
+      <c r="H4" s="156">
         <f>SUM(G4:G10)</f>
         <v>1641500</v>
       </c>
     </row>
-    <row r="5" s="94" customFormat="1" ht="40" customHeight="1" spans="1:8">
-      <c r="A5" s="112"/>
-      <c r="B5" s="113"/>
-      <c r="C5" s="119" t="s">
+    <row r="5" s="95" customFormat="1" ht="40" customHeight="1" spans="1:8">
+      <c r="A5" s="113"/>
+      <c r="B5" s="114"/>
+      <c r="C5" s="120" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="119">
+      <c r="D5" s="120">
         <v>100</v>
       </c>
-      <c r="E5" s="136"/>
-      <c r="F5" s="157">
+      <c r="E5" s="137"/>
+      <c r="F5" s="158">
         <v>630</v>
       </c>
-      <c r="G5" s="155">
+      <c r="G5" s="156">
         <f>SUM(D5*F5)</f>
         <v>63000</v>
       </c>
-      <c r="H5" s="156"/>
-    </row>
-    <row r="6" s="94" customFormat="1" ht="40" customHeight="1" spans="1:8">
-      <c r="A6" s="112"/>
-      <c r="B6" s="113"/>
-      <c r="C6" s="119" t="s">
+      <c r="H5" s="157"/>
+    </row>
+    <row r="6" s="95" customFormat="1" ht="40" customHeight="1" spans="1:8">
+      <c r="A6" s="113"/>
+      <c r="B6" s="114"/>
+      <c r="C6" s="120" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="119">
+      <c r="D6" s="120">
         <v>36</v>
       </c>
-      <c r="E6" s="136"/>
-      <c r="F6" s="157">
+      <c r="E6" s="137"/>
+      <c r="F6" s="158">
         <f>G6/D6</f>
         <v>3166.66666666667</v>
       </c>
-      <c r="G6" s="155">
+      <c r="G6" s="156">
         <v>114000</v>
       </c>
-      <c r="H6" s="156"/>
-    </row>
-    <row r="7" s="94" customFormat="1" ht="40" customHeight="1" spans="1:8">
-      <c r="A7" s="112"/>
-      <c r="B7" s="113"/>
-      <c r="C7" s="109" t="s">
+      <c r="H6" s="157"/>
+    </row>
+    <row r="7" s="95" customFormat="1" ht="40" customHeight="1" spans="1:8">
+      <c r="A7" s="113"/>
+      <c r="B7" s="114"/>
+      <c r="C7" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="109">
+      <c r="D7" s="110">
         <v>36</v>
       </c>
-      <c r="E7" s="136"/>
-      <c r="F7" s="157">
+      <c r="E7" s="137"/>
+      <c r="F7" s="158">
         <f>G7/D7</f>
         <v>2666.66666666667</v>
       </c>
-      <c r="G7" s="155">
+      <c r="G7" s="156">
         <v>96000</v>
       </c>
-      <c r="H7" s="156"/>
-    </row>
-    <row r="8" s="94" customFormat="1" ht="40" customHeight="1" spans="1:8">
-      <c r="A8" s="112"/>
-      <c r="B8" s="113"/>
-      <c r="C8" s="109" t="s">
+      <c r="H7" s="157"/>
+    </row>
+    <row r="8" s="95" customFormat="1" ht="40" customHeight="1" spans="1:8">
+      <c r="A8" s="113"/>
+      <c r="B8" s="114"/>
+      <c r="C8" s="110" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="109">
+      <c r="D8" s="110">
         <v>10</v>
       </c>
-      <c r="E8" s="136"/>
-      <c r="F8" s="157">
+      <c r="E8" s="137"/>
+      <c r="F8" s="158">
         <v>23000</v>
       </c>
-      <c r="G8" s="155">
+      <c r="G8" s="156">
         <f>F8*D8</f>
         <v>230000</v>
       </c>
-      <c r="H8" s="156"/>
-    </row>
-    <row r="9" s="94" customFormat="1" ht="40" customHeight="1" spans="1:8">
-      <c r="A9" s="112"/>
-      <c r="B9" s="113"/>
-      <c r="C9" s="109" t="s">
+      <c r="H8" s="157"/>
+    </row>
+    <row r="9" s="95" customFormat="1" ht="40" customHeight="1" spans="1:8">
+      <c r="A9" s="113"/>
+      <c r="B9" s="114"/>
+      <c r="C9" s="110" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="109">
+      <c r="D9" s="110">
         <v>7</v>
       </c>
-      <c r="E9" s="136"/>
-      <c r="F9" s="157">
+      <c r="E9" s="137"/>
+      <c r="F9" s="158">
         <f>G9/D9</f>
         <v>38000</v>
       </c>
-      <c r="G9" s="155">
+      <c r="G9" s="156">
         <v>266000</v>
       </c>
-      <c r="H9" s="156"/>
-    </row>
-    <row r="10" s="94" customFormat="1" ht="40" customHeight="1" spans="1:8">
-      <c r="A10" s="112"/>
-      <c r="B10" s="113"/>
-      <c r="C10" s="109" t="s">
+      <c r="H9" s="157"/>
+    </row>
+    <row r="10" s="95" customFormat="1" ht="40" customHeight="1" spans="1:8">
+      <c r="A10" s="113"/>
+      <c r="B10" s="114"/>
+      <c r="C10" s="110" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="109">
+      <c r="D10" s="110">
         <v>5</v>
       </c>
-      <c r="E10" s="136"/>
-      <c r="F10" s="157">
+      <c r="E10" s="137"/>
+      <c r="F10" s="158">
         <f>G10/D10</f>
         <v>12500</v>
       </c>
-      <c r="G10" s="155">
+      <c r="G10" s="156">
         <v>62500</v>
       </c>
-      <c r="H10" s="156"/>
-    </row>
-    <row r="11" s="94" customFormat="1" ht="258" customHeight="1" spans="1:8">
-      <c r="A11" s="116"/>
-      <c r="B11" s="119"/>
-      <c r="C11" s="119"/>
-      <c r="D11" s="119"/>
-      <c r="E11" s="139"/>
-      <c r="F11" s="158"/>
-      <c r="G11" s="154">
+      <c r="H10" s="157"/>
+    </row>
+    <row r="11" s="95" customFormat="1" ht="258" customHeight="1" spans="1:8">
+      <c r="A11" s="117"/>
+      <c r="B11" s="120"/>
+      <c r="C11" s="120"/>
+      <c r="D11" s="120"/>
+      <c r="E11" s="140"/>
+      <c r="F11" s="159"/>
+      <c r="G11" s="155">
         <f>SUM(D11*F11)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="154">
+      <c r="H11" s="155">
         <f>SUM(G11)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="12" s="94" customFormat="1" ht="18" customHeight="1" spans="1:8">
-      <c r="A12" s="152" t="s">
+    <row r="12" s="95" customFormat="1" ht="18" customHeight="1" spans="1:8">
+      <c r="A12" s="153" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="153"/>
-      <c r="C12" s="153"/>
-      <c r="D12" s="153"/>
-      <c r="E12" s="153"/>
-      <c r="F12" s="153"/>
-      <c r="G12" s="159"/>
-      <c r="H12" s="160">
+      <c r="B12" s="154"/>
+      <c r="C12" s="154"/>
+      <c r="D12" s="154"/>
+      <c r="E12" s="154"/>
+      <c r="F12" s="154"/>
+      <c r="G12" s="160"/>
+      <c r="H12" s="161">
         <f>SUM(H2:H11)</f>
         <v>3291500</v>
       </c>
@@ -2625,382 +2661,382 @@
   <dimension ref="A1:H19"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="20.4" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="19.859375" style="96"/>
-    <col min="2" max="2" width="21.6875" style="96" customWidth="1"/>
-    <col min="3" max="3" width="43.0390625" style="97" customWidth="1"/>
-    <col min="4" max="4" width="14.4296875" style="96" customWidth="1"/>
-    <col min="5" max="5" width="58.9609375" style="98" customWidth="1"/>
-    <col min="6" max="6" width="19.5234375" style="99" customWidth="1"/>
-    <col min="7" max="7" width="20.859375" style="99" customWidth="1"/>
-    <col min="8" max="8" width="20.859375" style="100" customWidth="1"/>
-    <col min="9" max="9" width="12.859375" style="98"/>
-    <col min="10" max="16384" width="9.140625" style="98"/>
+    <col min="1" max="1" width="19.859375" style="97"/>
+    <col min="2" max="2" width="21.6875" style="97" customWidth="1"/>
+    <col min="3" max="3" width="43.0390625" style="98" customWidth="1"/>
+    <col min="4" max="4" width="14.4296875" style="97" customWidth="1"/>
+    <col min="5" max="5" width="58.9609375" style="99" customWidth="1"/>
+    <col min="6" max="6" width="19.5234375" style="100" customWidth="1"/>
+    <col min="7" max="7" width="20.859375" style="100" customWidth="1"/>
+    <col min="8" max="8" width="20.859375" style="101" customWidth="1"/>
+    <col min="9" max="9" width="12.859375" style="99"/>
+    <col min="10" max="16384" width="9.140625" style="99"/>
   </cols>
   <sheetData>
-    <row r="1" s="94" customFormat="1" ht="16" customHeight="1" spans="1:8">
-      <c r="A1" s="101" t="s">
+    <row r="1" s="95" customFormat="1" ht="16" customHeight="1" spans="1:8">
+      <c r="A1" s="102" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="102" t="s">
+      <c r="B1" s="103" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="102" t="s">
+      <c r="C1" s="103" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="102" t="s">
+      <c r="D1" s="103" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="102" t="s">
+      <c r="E1" s="103" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="128" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="127" t="s">
+      <c r="G1" s="128" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="128" t="s">
+      <c r="H1" s="129" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" s="94" customFormat="1" ht="130" customHeight="1" spans="1:8">
-      <c r="A2" s="103">
+    <row r="2" s="95" customFormat="1" ht="130" customHeight="1" spans="1:8">
+      <c r="A2" s="104">
         <v>46055</v>
       </c>
-      <c r="B2" s="104" t="s">
+      <c r="B2" s="105" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="105" t="s">
+      <c r="C2" s="106" t="s">
         <v>19</v>
       </c>
       <c r="D2" s="20">
         <v>2</v>
       </c>
-      <c r="E2" s="104"/>
-      <c r="F2" s="129">
+      <c r="E2" s="105"/>
+      <c r="F2" s="130">
         <v>360000</v>
       </c>
-      <c r="G2" s="129">
+      <c r="G2" s="130">
         <f>D2*F2</f>
         <v>720000</v>
       </c>
-      <c r="H2" s="130">
+      <c r="H2" s="131">
         <f>SUM(G2:G3)</f>
         <v>870000</v>
       </c>
     </row>
-    <row r="3" s="94" customFormat="1" ht="130" customHeight="1" spans="1:8">
-      <c r="A3" s="106"/>
-      <c r="B3" s="107"/>
-      <c r="C3" s="105" t="s">
+    <row r="3" s="95" customFormat="1" ht="130" customHeight="1" spans="1:8">
+      <c r="A3" s="107"/>
+      <c r="B3" s="108"/>
+      <c r="C3" s="106" t="s">
         <v>20</v>
       </c>
       <c r="D3" s="20">
         <v>6</v>
       </c>
-      <c r="E3" s="107"/>
-      <c r="F3" s="129">
+      <c r="E3" s="108"/>
+      <c r="F3" s="130">
         <v>25000</v>
       </c>
-      <c r="G3" s="129">
+      <c r="G3" s="130">
         <f>D3*F3</f>
         <v>150000</v>
       </c>
-      <c r="H3" s="131"/>
-    </row>
-    <row r="4" s="94" customFormat="1" ht="130" customHeight="1" spans="1:8">
-      <c r="A4" s="108">
+      <c r="H3" s="132"/>
+    </row>
+    <row r="4" s="95" customFormat="1" ht="130" customHeight="1" spans="1:8">
+      <c r="A4" s="109">
         <v>46056</v>
       </c>
-      <c r="B4" s="109" t="s">
+      <c r="B4" s="110" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="110" t="s">
+      <c r="C4" s="111" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="111">
+      <c r="D4" s="112">
         <v>3</v>
       </c>
-      <c r="E4" s="132"/>
-      <c r="F4" s="133">
+      <c r="E4" s="133"/>
+      <c r="F4" s="134">
         <v>45000</v>
       </c>
-      <c r="G4" s="134">
+      <c r="G4" s="135">
         <f>D4*F4</f>
         <v>135000</v>
       </c>
-      <c r="H4" s="135">
+      <c r="H4" s="136">
         <f>SUM(G4:G5)</f>
         <v>515000</v>
       </c>
     </row>
-    <row r="5" s="94" customFormat="1" ht="130" customHeight="1" spans="1:8">
-      <c r="A5" s="112"/>
-      <c r="B5" s="113"/>
-      <c r="C5" s="114" t="s">
+    <row r="5" s="95" customFormat="1" ht="130" customHeight="1" spans="1:8">
+      <c r="A5" s="113"/>
+      <c r="B5" s="114"/>
+      <c r="C5" s="115" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="115">
+      <c r="D5" s="116">
         <v>10</v>
       </c>
-      <c r="E5" s="136"/>
-      <c r="F5" s="135">
+      <c r="E5" s="137"/>
+      <c r="F5" s="136">
         <v>38000</v>
       </c>
-      <c r="G5" s="135">
+      <c r="G5" s="136">
         <f>D5*F5</f>
         <v>380000</v>
       </c>
-      <c r="H5" s="137"/>
-    </row>
-    <row r="6" s="95" customFormat="1" ht="208.9" customHeight="1" spans="1:8">
-      <c r="A6" s="116">
+      <c r="H5" s="138"/>
+    </row>
+    <row r="6" s="96" customFormat="1" ht="208.9" customHeight="1" spans="1:8">
+      <c r="A6" s="117">
         <v>46066</v>
       </c>
-      <c r="B6" s="117" t="s">
+      <c r="B6" s="118" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="118" t="s">
+      <c r="C6" s="119" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="111">
+      <c r="D6" s="112">
         <v>3</v>
       </c>
-      <c r="E6" s="138"/>
-      <c r="F6" s="134">
+      <c r="E6" s="139"/>
+      <c r="F6" s="135">
         <v>75000</v>
       </c>
-      <c r="G6" s="134">
+      <c r="G6" s="135">
         <f>D6*F6</f>
         <v>225000</v>
       </c>
-      <c r="H6" s="134">
+      <c r="H6" s="135">
         <f>SUM(G6)</f>
         <v>225000</v>
       </c>
     </row>
-    <row r="7" s="95" customFormat="1" ht="70" customHeight="1" spans="1:8">
-      <c r="A7" s="116">
+    <row r="7" s="96" customFormat="1" ht="70" customHeight="1" spans="1:8">
+      <c r="A7" s="117">
         <v>46069</v>
       </c>
-      <c r="B7" s="119" t="s">
+      <c r="B7" s="120" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="118" t="s">
+      <c r="C7" s="119" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="111">
+      <c r="D7" s="112">
         <v>40</v>
       </c>
-      <c r="E7" s="139"/>
-      <c r="F7" s="134">
+      <c r="E7" s="140"/>
+      <c r="F7" s="135">
         <v>35000</v>
       </c>
-      <c r="G7" s="134">
+      <c r="G7" s="135">
         <f t="shared" ref="G7:G14" si="0">F7*D7</f>
         <v>1400000</v>
       </c>
-      <c r="H7" s="134">
+      <c r="H7" s="135">
         <f>SUM(G7:G9)</f>
         <v>5920000</v>
       </c>
     </row>
-    <row r="8" s="95" customFormat="1" ht="70" customHeight="1" spans="1:8">
-      <c r="A8" s="116"/>
-      <c r="B8" s="119"/>
-      <c r="C8" s="118" t="s">
+    <row r="8" s="96" customFormat="1" ht="70" customHeight="1" spans="1:8">
+      <c r="A8" s="117"/>
+      <c r="B8" s="120"/>
+      <c r="C8" s="119" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="111">
+      <c r="D8" s="112">
         <v>40</v>
       </c>
-      <c r="E8" s="139"/>
-      <c r="F8" s="134">
+      <c r="E8" s="140"/>
+      <c r="F8" s="135">
         <v>75000</v>
       </c>
-      <c r="G8" s="134">
+      <c r="G8" s="135">
         <f t="shared" si="0"/>
         <v>3000000</v>
       </c>
-      <c r="H8" s="134"/>
-    </row>
-    <row r="9" s="95" customFormat="1" ht="70" customHeight="1" spans="1:8">
-      <c r="A9" s="116"/>
-      <c r="B9" s="119"/>
-      <c r="C9" s="118" t="s">
+      <c r="H8" s="135"/>
+    </row>
+    <row r="9" s="96" customFormat="1" ht="70" customHeight="1" spans="1:8">
+      <c r="A9" s="117"/>
+      <c r="B9" s="120"/>
+      <c r="C9" s="119" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="111">
+      <c r="D9" s="112">
         <v>40</v>
       </c>
-      <c r="E9" s="139"/>
-      <c r="F9" s="134">
+      <c r="E9" s="140"/>
+      <c r="F9" s="135">
         <v>38000</v>
       </c>
-      <c r="G9" s="134">
+      <c r="G9" s="135">
         <f t="shared" si="0"/>
         <v>1520000</v>
       </c>
-      <c r="H9" s="134"/>
-    </row>
-    <row r="10" s="94" customFormat="1" ht="211.1" customHeight="1" spans="1:8">
-      <c r="A10" s="120">
+      <c r="H9" s="135"/>
+    </row>
+    <row r="10" s="95" customFormat="1" ht="211.1" customHeight="1" spans="1:8">
+      <c r="A10" s="121">
         <v>46070</v>
       </c>
-      <c r="B10" s="121" t="s">
+      <c r="B10" s="122" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="122" t="s">
+      <c r="C10" s="123" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="123">
+      <c r="D10" s="124">
         <v>2</v>
       </c>
-      <c r="E10" s="140"/>
-      <c r="F10" s="141">
+      <c r="E10" s="141"/>
+      <c r="F10" s="142">
         <v>295000</v>
       </c>
-      <c r="G10" s="141">
+      <c r="G10" s="142">
         <f t="shared" si="0"/>
         <v>590000</v>
       </c>
-      <c r="H10" s="141">
+      <c r="H10" s="142">
         <f>SUM(G10)</f>
         <v>590000</v>
       </c>
     </row>
-    <row r="11" s="94" customFormat="1" ht="55" customHeight="1" spans="1:8">
-      <c r="A11" s="112">
+    <row r="11" s="95" customFormat="1" ht="55" customHeight="1" spans="1:8">
+      <c r="A11" s="113">
         <v>46076</v>
       </c>
-      <c r="B11" s="113" t="s">
+      <c r="B11" s="114" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="122" t="s">
+      <c r="C11" s="123" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="111">
+      <c r="D11" s="112">
         <v>10</v>
       </c>
-      <c r="E11" s="136"/>
-      <c r="F11" s="134">
+      <c r="E11" s="137"/>
+      <c r="F11" s="135">
         <v>35000</v>
       </c>
-      <c r="G11" s="141">
+      <c r="G11" s="142">
         <f t="shared" si="0"/>
         <v>350000</v>
       </c>
-      <c r="H11" s="142">
+      <c r="H11" s="143">
         <f>SUM(G11:G14)</f>
         <v>1955000</v>
       </c>
     </row>
-    <row r="12" s="94" customFormat="1" ht="55" customHeight="1" spans="1:8">
-      <c r="A12" s="112"/>
-      <c r="B12" s="113"/>
-      <c r="C12" s="122" t="s">
+    <row r="12" s="95" customFormat="1" ht="55" customHeight="1" spans="1:8">
+      <c r="A12" s="113"/>
+      <c r="B12" s="114"/>
+      <c r="C12" s="123" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="111">
+      <c r="D12" s="112">
         <v>10</v>
       </c>
-      <c r="E12" s="136"/>
-      <c r="F12" s="134">
+      <c r="E12" s="137"/>
+      <c r="F12" s="135">
         <v>50000</v>
       </c>
-      <c r="G12" s="141">
+      <c r="G12" s="142">
         <f t="shared" si="0"/>
         <v>500000</v>
       </c>
-      <c r="H12" s="142"/>
-    </row>
-    <row r="13" s="94" customFormat="1" ht="55" customHeight="1" spans="1:8">
-      <c r="A13" s="112"/>
-      <c r="B13" s="113"/>
-      <c r="C13" s="122" t="s">
+      <c r="H12" s="143"/>
+    </row>
+    <row r="13" s="95" customFormat="1" ht="55" customHeight="1" spans="1:8">
+      <c r="A13" s="113"/>
+      <c r="B13" s="114"/>
+      <c r="C13" s="123" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="111">
+      <c r="D13" s="112">
         <v>500</v>
       </c>
-      <c r="E13" s="136"/>
-      <c r="F13" s="134">
+      <c r="E13" s="137"/>
+      <c r="F13" s="135">
         <v>2000</v>
       </c>
-      <c r="G13" s="141">
+      <c r="G13" s="142">
         <f t="shared" si="0"/>
         <v>1000000</v>
       </c>
-      <c r="H13" s="142"/>
-    </row>
-    <row r="14" s="94" customFormat="1" ht="55" customHeight="1" spans="1:8">
-      <c r="A14" s="120"/>
-      <c r="B14" s="124"/>
-      <c r="C14" s="122" t="s">
+      <c r="H13" s="143"/>
+    </row>
+    <row r="14" s="95" customFormat="1" ht="55" customHeight="1" spans="1:8">
+      <c r="A14" s="121"/>
+      <c r="B14" s="125"/>
+      <c r="C14" s="123" t="s">
         <v>36</v>
       </c>
-      <c r="D14" s="111">
+      <c r="D14" s="112">
         <v>3</v>
       </c>
-      <c r="E14" s="143"/>
-      <c r="F14" s="134">
+      <c r="E14" s="144"/>
+      <c r="F14" s="135">
         <v>35000</v>
       </c>
-      <c r="G14" s="141">
+      <c r="G14" s="142">
         <f t="shared" si="0"/>
         <v>105000</v>
       </c>
-      <c r="H14" s="144"/>
-    </row>
-    <row r="15" s="94" customFormat="1" spans="1:8">
-      <c r="A15" s="120"/>
-      <c r="B15" s="121"/>
-      <c r="C15" s="122"/>
-      <c r="D15" s="111"/>
-      <c r="E15" s="140"/>
-      <c r="F15" s="134"/>
-      <c r="G15" s="134"/>
-      <c r="H15" s="141"/>
-    </row>
-    <row r="16" s="94" customFormat="1" spans="1:8">
-      <c r="A16" s="120"/>
-      <c r="B16" s="121"/>
-      <c r="C16" s="122"/>
-      <c r="D16" s="111"/>
-      <c r="E16" s="140"/>
-      <c r="F16" s="134"/>
-      <c r="G16" s="134"/>
-      <c r="H16" s="141"/>
-    </row>
-    <row r="17" s="94" customFormat="1" spans="1:8">
-      <c r="A17" s="120"/>
-      <c r="B17" s="121"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="111"/>
-      <c r="E17" s="140"/>
-      <c r="F17" s="134"/>
-      <c r="G17" s="134"/>
-      <c r="H17" s="141"/>
-    </row>
-    <row r="18" s="94" customFormat="1" spans="1:8">
-      <c r="A18" s="120"/>
-      <c r="B18" s="124"/>
-      <c r="C18" s="122"/>
-      <c r="D18" s="111"/>
-      <c r="E18" s="143"/>
-      <c r="F18" s="133"/>
-      <c r="G18" s="134"/>
-      <c r="H18" s="141"/>
-    </row>
-    <row r="19" s="94" customFormat="1" spans="1:8">
-      <c r="A19" s="125"/>
-      <c r="B19" s="125"/>
-      <c r="C19" s="126"/>
-      <c r="D19" s="125"/>
-      <c r="E19" s="125"/>
-      <c r="F19" s="145"/>
-      <c r="G19" s="146"/>
-      <c r="H19" s="146">
+      <c r="H14" s="145"/>
+    </row>
+    <row r="15" s="95" customFormat="1" spans="1:8">
+      <c r="A15" s="121"/>
+      <c r="B15" s="122"/>
+      <c r="C15" s="123"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="141"/>
+      <c r="F15" s="135"/>
+      <c r="G15" s="135"/>
+      <c r="H15" s="142"/>
+    </row>
+    <row r="16" s="95" customFormat="1" spans="1:8">
+      <c r="A16" s="121"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="123"/>
+      <c r="D16" s="112"/>
+      <c r="E16" s="141"/>
+      <c r="F16" s="135"/>
+      <c r="G16" s="135"/>
+      <c r="H16" s="142"/>
+    </row>
+    <row r="17" s="95" customFormat="1" spans="1:8">
+      <c r="A17" s="121"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="123"/>
+      <c r="D17" s="112"/>
+      <c r="E17" s="141"/>
+      <c r="F17" s="135"/>
+      <c r="G17" s="135"/>
+      <c r="H17" s="142"/>
+    </row>
+    <row r="18" s="95" customFormat="1" spans="1:8">
+      <c r="A18" s="121"/>
+      <c r="B18" s="125"/>
+      <c r="C18" s="123"/>
+      <c r="D18" s="112"/>
+      <c r="E18" s="144"/>
+      <c r="F18" s="134"/>
+      <c r="G18" s="135"/>
+      <c r="H18" s="142"/>
+    </row>
+    <row r="19" s="95" customFormat="1" spans="1:8">
+      <c r="A19" s="126"/>
+      <c r="B19" s="126"/>
+      <c r="C19" s="127"/>
+      <c r="D19" s="126"/>
+      <c r="E19" s="126"/>
+      <c r="F19" s="146"/>
+      <c r="G19" s="147"/>
+      <c r="H19" s="147">
         <f>SUM(H2:H18)</f>
         <v>10075000</v>
       </c>
@@ -3074,7 +3110,7 @@
       <c r="A2" s="61">
         <v>46055</v>
       </c>
-      <c r="B2" s="47" t="s">
+      <c r="B2" s="49" t="s">
         <v>37</v>
       </c>
       <c r="C2" s="62" t="s">
@@ -3094,7 +3130,7 @@
     </row>
     <row r="3" ht="191" customHeight="1" spans="1:7">
       <c r="A3" s="61"/>
-      <c r="B3" s="47"/>
+      <c r="B3" s="49"/>
       <c r="C3" s="64"/>
       <c r="D3" s="65"/>
       <c r="E3" s="79"/>
@@ -3114,7 +3150,7 @@
         <f>SUM(G2:G3)</f>
         <v>485117.056</v>
       </c>
-      <c r="I4" s="93"/>
+      <c r="I4" s="94"/>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="61"/>
@@ -3129,7 +3165,7 @@
         <f>G4*11%</f>
         <v>53362.87616</v>
       </c>
-      <c r="I5" s="93"/>
+      <c r="I5" s="94"/>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="61"/>
@@ -3172,8 +3208,8 @@
       <c r="D8" s="70">
         <v>120</v>
       </c>
-      <c r="E8" s="49"/>
-      <c r="F8" s="87">
+      <c r="E8" s="87"/>
+      <c r="F8" s="88">
         <v>6063.9632</v>
       </c>
       <c r="G8" s="81">
@@ -3188,7 +3224,7 @@
       </c>
       <c r="C9" s="66"/>
       <c r="D9" s="67"/>
-      <c r="E9" s="88"/>
+      <c r="E9" s="89"/>
       <c r="F9" s="83"/>
       <c r="G9" s="84">
         <f>SUM(G8:G8)</f>
@@ -3202,7 +3238,7 @@
       </c>
       <c r="C10" s="71"/>
       <c r="D10" s="67"/>
-      <c r="E10" s="88"/>
+      <c r="E10" s="89"/>
       <c r="F10" s="83"/>
       <c r="G10" s="84">
         <f>G9*11%</f>
@@ -3216,7 +3252,7 @@
       </c>
       <c r="C11" s="66"/>
       <c r="D11" s="67"/>
-      <c r="E11" s="88"/>
+      <c r="E11" s="89"/>
       <c r="F11" s="83"/>
       <c r="G11" s="84">
         <f>((G9*100)/111)*0.111%</f>
@@ -3231,7 +3267,7 @@
       <c r="C12" s="74"/>
       <c r="D12" s="67"/>
       <c r="E12" s="85"/>
-      <c r="F12" s="89"/>
+      <c r="F12" s="90"/>
       <c r="G12" s="84">
         <f>SUM(G9:G11)</f>
         <v>808447.573824</v>
@@ -3244,12 +3280,11 @@
       <c r="B13" s="76"/>
       <c r="C13" s="76"/>
       <c r="D13" s="77"/>
-      <c r="E13" s="90">
-        <f>G7+G12</f>
-        <v>1347412.62304</v>
-      </c>
-      <c r="F13" s="91"/>
-      <c r="G13" s="92"/>
+      <c r="E13" s="91">
+        <v>1347412</v>
+      </c>
+      <c r="F13" s="92"/>
+      <c r="G13" s="93"/>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -3281,262 +3316,411 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E32"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelCol="4"/>
+  <dimension ref="A1:D28"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="10.5703125" style="12" customWidth="1"/>
     <col min="2" max="2" width="12.6015625" style="44" customWidth="1"/>
-    <col min="3" max="3" width="36.125" style="12" customWidth="1"/>
-    <col min="4" max="4" width="18.828125" style="12" customWidth="1"/>
-    <col min="5" max="5" width="12.2890625" style="12" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="12"/>
+    <col min="3" max="3" width="18.828125" style="12" customWidth="1"/>
+    <col min="4" max="4" width="12.2890625" style="45" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" s="43" customFormat="1" ht="19" customHeight="1" spans="1:5">
-      <c r="A1" s="45" t="s">
+    <row r="1" s="43" customFormat="1" ht="26" spans="1:4">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="45" t="s">
+      <c r="C1" s="46" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="48" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" s="12" customFormat="1" spans="1:4">
+      <c r="A2" s="49">
+        <v>46054</v>
+      </c>
+      <c r="B2" s="50">
+        <v>1490</v>
+      </c>
+      <c r="C2" s="51">
+        <f>64000</f>
+        <v>64000</v>
+      </c>
+      <c r="D2" s="52">
+        <f>C2/8000</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" s="12" customFormat="1" spans="1:4">
+      <c r="A3" s="49">
+        <v>46055</v>
+      </c>
+      <c r="B3" s="50">
+        <v>1491</v>
+      </c>
+      <c r="C3" s="53">
+        <v>48000</v>
+      </c>
+      <c r="D3" s="52">
+        <f t="shared" ref="D3:D25" si="0">C3/8000</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" s="12" customFormat="1" spans="1:4">
+      <c r="A4" s="49">
+        <v>46056</v>
+      </c>
+      <c r="B4" s="50">
+        <v>1492</v>
+      </c>
+      <c r="C4" s="53">
+        <v>24000</v>
+      </c>
+      <c r="D4" s="52">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" s="12" customFormat="1" spans="1:4">
+      <c r="A5" s="49">
+        <v>46057</v>
+      </c>
+      <c r="B5" s="50">
+        <v>1493</v>
+      </c>
+      <c r="C5" s="53">
+        <v>96000</v>
+      </c>
+      <c r="D5" s="52">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" s="12" customFormat="1" spans="1:4">
+      <c r="A6" s="49">
+        <v>46058</v>
+      </c>
+      <c r="B6" s="50">
+        <v>1494</v>
+      </c>
+      <c r="C6" s="53">
+        <v>8000</v>
+      </c>
+      <c r="D6" s="52">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" s="12" customFormat="1" spans="1:4">
+      <c r="A7" s="49">
+        <v>46060</v>
+      </c>
+      <c r="B7" s="50">
+        <v>1495</v>
+      </c>
+      <c r="C7" s="53">
+        <v>40000</v>
+      </c>
+      <c r="D7" s="52">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" s="12" customFormat="1" spans="1:4">
+      <c r="A8" s="49">
+        <v>46061</v>
+      </c>
+      <c r="B8" s="50">
+        <v>1496</v>
+      </c>
+      <c r="C8" s="53">
+        <v>24000</v>
+      </c>
+      <c r="D8" s="52">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" s="12" customFormat="1" spans="1:4">
+      <c r="A9" s="49">
+        <v>46062</v>
+      </c>
+      <c r="B9" s="50">
+        <v>1497</v>
+      </c>
+      <c r="C9" s="53">
+        <v>48000</v>
+      </c>
+      <c r="D9" s="52">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" s="12" customFormat="1" spans="1:4">
+      <c r="A10" s="49">
+        <v>46063</v>
+      </c>
+      <c r="B10" s="50">
+        <v>1498</v>
+      </c>
+      <c r="C10" s="53">
+        <v>24000</v>
+      </c>
+      <c r="D10" s="52">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" s="12" customFormat="1" spans="1:4">
+      <c r="A11" s="49">
+        <v>46064</v>
+      </c>
+      <c r="B11" s="50">
+        <v>1499</v>
+      </c>
+      <c r="C11" s="53">
+        <v>32000</v>
+      </c>
+      <c r="D11" s="52">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="D1" s="45" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="45" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" s="12" customFormat="1" ht="263.65" customHeight="1" spans="1:5">
-      <c r="A2" s="47"/>
-      <c r="B2" s="48"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="49"/>
-    </row>
-    <row r="3" s="12" customFormat="1" ht="255.1" customHeight="1" spans="1:5">
-      <c r="A3" s="47"/>
-      <c r="B3" s="48"/>
-      <c r="C3" s="49"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="56"/>
-    </row>
-    <row r="4" s="12" customFormat="1" ht="249.95" customHeight="1" spans="1:5">
-      <c r="A4" s="47"/>
-      <c r="B4" s="48"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="51"/>
-      <c r="E4" s="56"/>
-    </row>
-    <row r="5" s="12" customFormat="1" ht="256.25" customHeight="1" spans="1:5">
-      <c r="A5" s="47"/>
-      <c r="B5" s="48"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="51"/>
-      <c r="E5" s="56"/>
-    </row>
-    <row r="6" s="12" customFormat="1" ht="253.85" customHeight="1" spans="1:5">
-      <c r="A6" s="47"/>
-      <c r="B6" s="48"/>
-      <c r="C6" s="49"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="56"/>
-    </row>
-    <row r="7" s="12" customFormat="1" ht="254.65" customHeight="1" spans="1:5">
-      <c r="A7" s="47"/>
-      <c r="B7" s="48"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="51"/>
-      <c r="E7" s="56"/>
-    </row>
-    <row r="8" s="12" customFormat="1" ht="255.35" customHeight="1" spans="1:5">
-      <c r="A8" s="47"/>
-      <c r="B8" s="48"/>
-      <c r="C8" s="49"/>
-      <c r="D8" s="51"/>
-      <c r="E8" s="56"/>
-    </row>
-    <row r="9" s="12" customFormat="1" ht="266.95" customHeight="1" spans="1:5">
-      <c r="A9" s="47"/>
-      <c r="B9" s="48"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="51"/>
-      <c r="E9" s="56"/>
-    </row>
-    <row r="10" s="12" customFormat="1" ht="261.95" customHeight="1" spans="1:5">
-      <c r="A10" s="47"/>
-      <c r="B10" s="48"/>
-      <c r="C10" s="49"/>
-      <c r="D10" s="51"/>
-      <c r="E10" s="56"/>
-    </row>
-    <row r="11" s="12" customFormat="1" ht="261.9" customHeight="1" spans="1:5">
-      <c r="A11" s="47"/>
-      <c r="B11" s="48"/>
-      <c r="C11" s="49"/>
-      <c r="D11" s="51"/>
-      <c r="E11" s="56"/>
-    </row>
-    <row r="12" s="12" customFormat="1" ht="270.7" customHeight="1" spans="1:5">
-      <c r="A12" s="47"/>
-      <c r="B12" s="48"/>
-      <c r="C12" s="49"/>
-      <c r="D12" s="51"/>
-      <c r="E12" s="56"/>
-    </row>
-    <row r="13" s="12" customFormat="1" ht="261.1" customHeight="1" spans="1:5">
-      <c r="A13" s="47"/>
-      <c r="B13" s="48"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="51"/>
-      <c r="E13" s="56"/>
-    </row>
-    <row r="14" s="12" customFormat="1" ht="257.15" customHeight="1" spans="1:5">
-      <c r="A14" s="47"/>
-      <c r="B14" s="48"/>
-      <c r="C14" s="49"/>
-      <c r="D14" s="51"/>
-      <c r="E14" s="56"/>
-    </row>
-    <row r="15" s="12" customFormat="1" ht="263.55" customHeight="1" spans="1:5">
-      <c r="A15" s="47"/>
-      <c r="B15" s="48"/>
-      <c r="C15" s="49"/>
-      <c r="D15" s="51"/>
-      <c r="E15" s="56"/>
-    </row>
-    <row r="16" s="12" customFormat="1" ht="270.35" customHeight="1" spans="1:5">
-      <c r="A16" s="47"/>
-      <c r="B16" s="48"/>
-      <c r="C16" s="49"/>
-      <c r="D16" s="51"/>
-      <c r="E16" s="56"/>
-    </row>
-    <row r="17" s="12" customFormat="1" ht="261.7" customHeight="1" spans="1:5">
-      <c r="A17" s="47"/>
-      <c r="B17" s="48"/>
-      <c r="C17" s="49"/>
-      <c r="D17" s="51"/>
-      <c r="E17" s="56"/>
-    </row>
-    <row r="18" s="12" customFormat="1" ht="260" customHeight="1" spans="1:5">
-      <c r="A18" s="47"/>
-      <c r="B18" s="48"/>
-      <c r="C18" s="49"/>
-      <c r="D18" s="51"/>
-      <c r="E18" s="56"/>
-    </row>
-    <row r="19" s="12" customFormat="1" ht="263.2" customHeight="1" spans="1:5">
-      <c r="A19" s="47"/>
-      <c r="B19" s="48"/>
-      <c r="C19" s="49"/>
-      <c r="D19" s="51"/>
-      <c r="E19" s="56"/>
-    </row>
-    <row r="20" s="12" customFormat="1" ht="289.95" customHeight="1" spans="1:5">
-      <c r="A20" s="47"/>
-      <c r="B20" s="48"/>
-      <c r="C20" s="49"/>
-      <c r="D20" s="51"/>
-      <c r="E20" s="56"/>
-    </row>
-    <row r="21" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A21" s="47"/>
-      <c r="B21" s="48"/>
-      <c r="C21" s="49"/>
-      <c r="D21" s="51"/>
-      <c r="E21" s="56"/>
-    </row>
-    <row r="22" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A22" s="47"/>
-      <c r="B22" s="48"/>
-      <c r="C22" s="49"/>
-      <c r="D22" s="51"/>
-      <c r="E22" s="56"/>
-    </row>
-    <row r="23" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A23" s="47"/>
-      <c r="B23" s="48"/>
-      <c r="C23" s="49"/>
-      <c r="D23" s="51"/>
-      <c r="E23" s="56"/>
-    </row>
-    <row r="24" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A24" s="47"/>
-      <c r="B24" s="48"/>
-      <c r="C24" s="49"/>
-      <c r="D24" s="50"/>
-      <c r="E24" s="49"/>
-    </row>
-    <row r="25" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A25" s="47"/>
-      <c r="B25" s="48"/>
-      <c r="C25" s="49"/>
-      <c r="D25" s="50"/>
-      <c r="E25" s="49"/>
-    </row>
-    <row r="26" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A26" s="47"/>
-      <c r="B26" s="48"/>
-      <c r="C26" s="49"/>
-      <c r="D26" s="50"/>
-      <c r="E26" s="49"/>
-    </row>
-    <row r="27" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A27" s="47">
-        <v>45960</v>
-      </c>
-      <c r="B27" s="48"/>
-      <c r="C27" s="49"/>
-      <c r="D27" s="50"/>
-      <c r="E27" s="49"/>
-    </row>
-    <row r="28" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A28" s="47">
-        <v>45961</v>
-      </c>
-      <c r="B28" s="48"/>
-      <c r="C28" s="49"/>
-      <c r="D28" s="50"/>
-      <c r="E28" s="49"/>
-    </row>
-    <row r="29" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A29" s="47"/>
-      <c r="B29" s="48"/>
-      <c r="C29" s="49"/>
-      <c r="D29" s="50"/>
-      <c r="E29" s="49"/>
-    </row>
-    <row r="30" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A30" s="47"/>
-      <c r="B30" s="48"/>
-      <c r="C30" s="49"/>
-      <c r="D30" s="50"/>
-      <c r="E30" s="49"/>
-    </row>
-    <row r="31" s="12" customFormat="1" ht="200" customHeight="1" spans="1:5">
-      <c r="A31" s="47"/>
-      <c r="B31" s="48"/>
-      <c r="C31" s="49"/>
-      <c r="D31" s="50"/>
-      <c r="E31" s="49"/>
-    </row>
-    <row r="32" s="12" customFormat="1" spans="1:5">
-      <c r="A32" s="52"/>
-      <c r="B32" s="53"/>
-      <c r="C32" s="54">
-        <f>SUM(D2:D31)</f>
+    </row>
+    <row r="12" s="12" customFormat="1" spans="1:4">
+      <c r="A12" s="49">
+        <v>46065</v>
+      </c>
+      <c r="B12" s="50">
+        <v>1500</v>
+      </c>
+      <c r="C12" s="53">
+        <v>40000</v>
+      </c>
+      <c r="D12" s="52">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" s="12" customFormat="1" spans="1:4">
+      <c r="A13" s="49">
+        <v>46066</v>
+      </c>
+      <c r="B13" s="162" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="53">
+        <v>48000</v>
+      </c>
+      <c r="D13" s="52">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" s="12" customFormat="1" spans="1:4">
+      <c r="A14" s="49">
+        <v>46067</v>
+      </c>
+      <c r="B14" s="162" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="53">
+        <v>40000</v>
+      </c>
+      <c r="D14" s="52">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" s="12" customFormat="1" spans="1:4">
+      <c r="A15" s="49">
+        <v>46068</v>
+      </c>
+      <c r="B15" s="162" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="53">
+        <v>40000</v>
+      </c>
+      <c r="D15" s="52">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" s="12" customFormat="1" spans="1:4">
+      <c r="A16" s="49">
+        <v>46069</v>
+      </c>
+      <c r="B16" s="162" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="53">
+        <v>40000</v>
+      </c>
+      <c r="D16" s="52">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" s="12" customFormat="1" spans="1:4">
+      <c r="A17" s="49">
+        <v>46070</v>
+      </c>
+      <c r="B17" s="162" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="53">
+        <v>32000</v>
+      </c>
+      <c r="D17" s="52">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" s="12" customFormat="1" spans="1:4">
+      <c r="A18" s="49">
+        <v>46072</v>
+      </c>
+      <c r="B18" s="162" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="53">
+        <v>88000</v>
+      </c>
+      <c r="D18" s="52">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" s="12" customFormat="1" spans="1:4">
+      <c r="A19" s="49">
+        <v>46074</v>
+      </c>
+      <c r="B19" s="162" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" s="53">
+        <v>24000</v>
+      </c>
+      <c r="D19" s="52">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" s="12" customFormat="1" spans="1:4">
+      <c r="A20" s="49">
+        <v>46076</v>
+      </c>
+      <c r="B20" s="162" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="51">
+        <v>110000</v>
+      </c>
+      <c r="D20" s="52">
+        <f t="shared" si="0"/>
+        <v>13.75</v>
+      </c>
+    </row>
+    <row r="21" s="12" customFormat="1" spans="1:4">
+      <c r="A21" s="49">
+        <v>46077</v>
+      </c>
+      <c r="B21" s="162" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" s="51">
+        <v>48000</v>
+      </c>
+      <c r="D21" s="52">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" s="12" customFormat="1" spans="1:4">
+      <c r="A22" s="49">
+        <v>46078</v>
+      </c>
+      <c r="B22" s="162" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="51">
+        <v>32000</v>
+      </c>
+      <c r="D22" s="52">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" s="12" customFormat="1" spans="1:4">
+      <c r="A23" s="49">
+        <v>46079</v>
+      </c>
+      <c r="B23" s="162" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="51">
+        <v>96000</v>
+      </c>
+      <c r="D23" s="52">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" s="12" customFormat="1" spans="1:4">
+      <c r="A24" s="49">
+        <v>46080</v>
+      </c>
+      <c r="B24" s="162" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="51">
+        <v>32000</v>
+      </c>
+      <c r="D24" s="52">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" s="12" customFormat="1" spans="1:4">
+      <c r="A25" s="49">
+        <v>46081</v>
+      </c>
+      <c r="B25" s="50"/>
+      <c r="C25" s="51"/>
+      <c r="D25" s="52">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D32" s="55"/>
-      <c r="E32" s="57"/>
+    </row>
+    <row r="26" s="12" customFormat="1" ht="200" customHeight="1" spans="1:4">
+      <c r="A26" s="49"/>
+      <c r="B26" s="50"/>
+      <c r="C26" s="51"/>
+      <c r="D26" s="52"/>
+    </row>
+    <row r="27" s="12" customFormat="1" ht="200" customHeight="1" spans="1:4">
+      <c r="A27" s="49"/>
+      <c r="B27" s="50"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="52"/>
+    </row>
+    <row r="28" s="12" customFormat="1" spans="1:4">
+      <c r="A28" s="54"/>
+      <c r="B28" s="55"/>
+      <c r="C28" s="56"/>
+      <c r="D28" s="57">
+        <f>SUM(C:C)</f>
+        <v>1078000</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C32:E32"/>
+  <mergeCells count="1">
+    <mergeCell ref="A28:B28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -3562,10 +3746,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D1" s="17" t="s">
         <v>4</v>
@@ -3585,7 +3769,7 @@
         <v>46056</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="C2" s="20">
         <v>5</v>
@@ -3608,7 +3792,7 @@
         <v>46069</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="C3" s="24">
         <v>10</v>
@@ -3629,7 +3813,7 @@
     <row r="4" s="12" customFormat="1" ht="150" customHeight="1" spans="1:7">
       <c r="A4" s="26"/>
       <c r="B4" s="27" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C4" s="24">
         <v>5</v>
@@ -3701,13 +3885,13 @@
   <sheetData>
     <row r="1" ht="25" customHeight="1" spans="1:3">
       <c r="A1" s="3" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -3715,7 +3899,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="C2" s="8">
         <f>'Anugrah (Bag, Cup, Box)'!H12</f>
@@ -3727,7 +3911,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="C3" s="8">
         <f>'UD Abdi Jaya (Bag, Cup, Box)'!H19</f>
@@ -3739,11 +3923,11 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="C4" s="8">
         <f>'PT. SUPARMA JAYA TBK (Tissue)'!E13</f>
-        <v>1347412.62304</v>
+        <v>1347412</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -3751,11 +3935,11 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="C5" s="9">
-        <f>'Vickel Laundry'!C32</f>
-        <v>0</v>
+        <f>'Vickel Laundry'!D28</f>
+        <v>1078000</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -3763,7 +3947,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="C6" s="9">
         <f>'Dishy Soap'!G7</f>
@@ -3777,7 +3961,7 @@
       <c r="B7" s="7"/>
       <c r="C7" s="10">
         <f>SUM(C2:C5)</f>
-        <v>14713912.62304</v>
+        <v>15791912</v>
       </c>
     </row>
   </sheetData>

</xml_diff>